<commit_message>
feat(P6): Prediction 8종 추가 + Feature 5종 삭제
Prediction 채움 (기존 문장 스타일 + [Confidence] + Branch)
- Late Arm, Trail Elbow Behind Body(2분기), Steep Shaft(2분기), Shallow Shaft,
  Casting, Lead Pressure Insufficient, Lead Pressure Excessive(2분기), Spin-out
- 남은 placeholder 2: Pelvis Stall / Incomplete Pressure Transfer (예측 미지정)

삭제 5 (중복/Evidence Layer로 흡수)
- Handle Raise, Handle Too Low, Spine Angle Loss, Late Trail Foot Release, Left Start Direction
- 삭제 노드는 체인에서 제거하고 앞뒤 연결 유지 (chain/cooc 정리)

신규 Prediction 어휘 등록 (prediction-vocab)
- Early Upper Body Rotation, Blocked Body Rotation, Trail Elbow Tucked, Reduced Lag,
  Thoracic Hyperextension, Increased Vertical Force, Side Bend Compensation,
  Excessive Side Bend, Trail Arm Extension Compensation

Evidence Matrix: 삭제 반영 (41→36 features)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015JSgPBxwLoJqyCWhXnBVL3
</commit_message>
<xml_diff>
--- a/DOH_P6.xlsx
+++ b/DOH_P6.xlsx
@@ -16,8 +16,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mechanism_Dictionary'!$A$1:$F$79</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Feature_Dictionary'!$A$1:$E$50</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Evidence Matrix'!$A$1:$O$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Feature_Dictionary'!$A$1:$E$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Evidence Matrix'!$A$1:$O$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'TODO'!$A$1:$E$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -908,9 +908,7 @@
 The Pelvis Rotates Faster Than The Arms Can Follow.
 (팔이 따라올 수 없을 만큼 골반이 빠르게 회전한다.)
    ↓
-Arm Stuck (팔 끼임)
-   ↓
-Handle Raise (핸들 상승)</t>
+Arm Stuck (팔 끼임)</t>
         </is>
       </c>
     </row>
@@ -988,8 +986,7 @@
         <is>
           <t>· Thorax Rotation Excessive (흉곽 과회전)
 · Spin-out (스핀아웃)
-· Club Face Open (클럽페이스 오픈)
-· Handle Raise (핸들 상승)</t>
+· Club Face Open (클럽페이스 오픈)</t>
         </is>
       </c>
     </row>
@@ -1404,7 +1401,14 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>(예측 정리 예정 — Evidence Matrix 참조)</t>
+          <t>[Medium Confidence]
+Spin-out (P6)
+   ↓
+Early Upper Body Rotation.
+   ↓
+Forward Hands.
+   ↓
+Steep Club Delivery.</t>
         </is>
       </c>
     </row>
@@ -1548,9 +1552,7 @@
           <t>Early Extension (얼리 익스텐션)
    ↓
 The Body Loses Delivery Space.
-(다운스윙 공간이 부족해진다.)
-   ↓
-Handle Raise (핸들 상승)</t>
+(다운스윙 공간이 부족해진다.)</t>
         </is>
       </c>
     </row>
@@ -2270,7 +2272,14 @@
       </c>
       <c r="B124" s="4" t="inlineStr">
         <is>
-          <t>(예측 정리 예정 — Evidence Matrix 참조)</t>
+          <t>[Medium Confidence]
+Lead Pressure Insufficient (P6)
+   ↓
+Early Upper Body Rotation.
+   ↓
+Forward Hands.
+   ↓
+Steep Club Delivery.</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2478,21 @@
       </c>
       <c r="B139" s="4" t="inlineStr">
         <is>
-          <t>(예측 정리 예정 — Evidence Matrix 참조)</t>
+          <t>[Pattern Dependent]
+Lead Pressure Excessive (P6)
+   ↓
+Blocked Body Rotation.
+   ↓
+Inside Club Delivery.
+──────────────────
+Lead Pressure Excessive (P6)
+   ↓
+Early Upper Body Rotation.
+   ↓
+Forward Hands.
+   ↓
+Steep Club Delivery.
+※ 양쪽 패턴 모두 존재 → Branch 유지.</t>
         </is>
       </c>
     </row>
@@ -2813,9 +2836,7 @@
           <t>Head Drop (머리 하강)
    ↓
 The Body Moves Toward The Ball And Loses Space.
-(몸이 볼 방향으로 이동하며 공간을 잃는다.)
-   ↓
-Handle Too Low (핸들 낮음)</t>
+(몸이 볼 방향으로 이동하며 공간을 잃는다.)</t>
         </is>
       </c>
     </row>
@@ -2892,7 +2913,6 @@
           <t>· Spine Flexion Excessive (척추 과굴곡)
 · Trail Side Bend Excessive (트레일측 측굴 과다)
 · Deep Hands (손 깊음)
-· Handle Too Low (핸들 낮음)
 · Hanging Back (체중 뒤잔류)
 · Club Face Closed (클럽페이스 클로즈)</t>
         </is>
@@ -3964,7 +3984,14 @@
       </c>
       <c r="B255" s="4" t="inlineStr">
         <is>
-          <t>(예측 정리 예정 — Evidence Matrix 참조)</t>
+          <t>[Medium Confidence]
+Late Arm (P6)
+   ↓
+Forward Hands.
+   ↓
+Steep Club Delivery.
+   ↓
+Club Face Open At Impact.</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4133,21 @@
       </c>
       <c r="B266" s="4" t="inlineStr">
         <is>
-          <t>(예측 정리 예정 — Evidence Matrix 참조)</t>
+          <t>[Pattern Dependent]
+Trail Elbow Behind Body (P6)
+   ↓
+Forward Hands.
+   ↓
+Steep Club Delivery.
+──────────────────
+Trail Elbow Behind Body (P6)
+   ↓
+Deep Hands.
+   ↓
+Casting.
+   ↓
+Inside Club Delivery.
+※ 뒤에 남는 패턴이 Forward Hands vs Deep Hands 두 갈래 → Branch 유지.</t>
         </is>
       </c>
     </row>
@@ -4309,7 +4350,19 @@
       </c>
       <c r="B282" s="4" t="inlineStr">
         <is>
-          <t>(예측 정리 예정 — Evidence Matrix 참조)</t>
+          <t>[Pattern Dependent]
+Steep Shaft (P6)
+   ↓
+Steep Club Delivery.
+   ↓
+Club Face Open At Impact.
+──────────────────
+Steep Shaft (P6)
+   ↓
+Trail Elbow Tucked.
+   ↓
+Club Face Closed At Impact.
+※ Steep인데도 훅이 나는 경우를 Branch로 처리.</t>
         </is>
       </c>
     </row>
@@ -4507,7 +4560,12 @@
       </c>
       <c r="B298" s="4" t="inlineStr">
         <is>
-          <t>(예측 정리 예정 — Evidence Matrix 참조)</t>
+          <t>[Medium Confidence]
+Shallow Shaft (P6)
+   ↓
+Inside Club Delivery.
+   ↓
+Club Face Closed At Impact.</t>
         </is>
       </c>
     </row>
@@ -4698,7 +4756,15 @@
       </c>
       <c r="B313" s="4" t="inlineStr">
         <is>
-          <t>(예측 정리 예정 — Evidence Matrix 참조)</t>
+          <t>[Medium Confidence]
+Casting (P6)
+   ↓
+Reduced Lag.
+   ↓
+Reduced Club Control.
+   ↓
+Club Face Open At Impact.
+※ Pull Slice도 결국 Face Control 실패로 귀결 — 이 수준에서 종료(DOH 스타일).</t>
         </is>
       </c>
     </row>
@@ -7213,7 +7279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -7895,111 +7961,111 @@
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t>Late Trail Foot Release</t>
+          <t>Cross-over Top Pattern</t>
         </is>
       </c>
       <c r="B25" s="13" t="inlineStr">
         <is>
-          <t>트레일발 이탈 지연</t>
+          <t>크로스오버 탑 패턴</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>다운스윙 전달 구간에서도 트레일발에 하중이 계속 남아 이탈이 지연되는 현상.</t>
+          <t>백스윙 탑(P4)에서 클럽이 스윙플레인을 넘어가는 패턴. Lead Pressure Excessive + Thoracic Hyperextension 복합에서 반복 관찰 — 독립 Feature보다 Composite Observation 후보.</t>
         </is>
       </c>
       <c r="D25" s="13" t="inlineStr">
         <is>
-          <t>Pressure</t>
+          <t>Club</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Timing, Trail
-[status] pending</t>
+          <t>P4, Composite
+[status] candidate-composite · 프로 메모</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>Left Start Direction</t>
+          <t>Spine Flexion Excessive</t>
         </is>
       </c>
       <c r="B26" s="13" t="inlineStr">
         <is>
-          <t>출발 방향 좌측</t>
+          <t>척추 과굴곡</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>임팩트에서 클럽 경로가 좌측으로 진행되어 볼 출발 방향이 좌측이 되는 결과.</t>
+          <t>다운스윙 중반(P6)에서 척추(흉요추)가 정상보다 과도하게 굴곡되어 상체가 숙여지는 현상. Spine Extension Excessive와 반대 방향.</t>
         </is>
       </c>
       <c r="D26" s="13" t="inlineStr">
         <is>
-          <t>Club</t>
+          <t>Spine</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Ball Flight
-[status] pending · Ball Flight Observation</t>
+          <t>Magnitude, Excessive
+[status] pending</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t>Cross-over Top Pattern</t>
+          <t>Trail Side Bend Excessive</t>
         </is>
       </c>
       <c r="B27" s="13" t="inlineStr">
         <is>
-          <t>크로스오버 탑 패턴</t>
+          <t>트레일측 측굴 과다</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>백스윙 탑(P4)에서 클럽이 스윙플레인을 넘어가는 패턴. Lead Pressure Excessive + Thoracic Hyperextension 복합에서 반복 관찰 — 독립 Feature보다 Composite Observation 후보.</t>
+          <t>다운스윙 중반(P6)에서 몸통의 트레일측 측면 굴곡이 정상보다 과도한 현상.</t>
         </is>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>Club</t>
+          <t>Thorax</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>P4, Composite
-[status] candidate-composite · 프로 메모</t>
+          <t>Magnitude, Excessive
+[status] pending</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t>Spine Flexion Excessive</t>
+          <t>Chicken Wing Pattern</t>
         </is>
       </c>
       <c r="B28" s="13" t="inlineStr">
         <is>
-          <t>척추 과굴곡</t>
+          <t>치킨윙 패턴</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>다운스윙 중반(P6)에서 척추(흉요추)가 정상보다 과도하게 굴곡되어 상체가 숙여지는 현상. Spine Extension Excessive와 반대 방향.</t>
+          <t>임팩트 구간에서 리드암이 충분히 신전되지 못하고 굽혀지는 패턴. 공간·전달 실패의 보상.</t>
         </is>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>Spine</t>
+          <t>Arm</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Magnitude, Excessive
+          <t>Pattern
 [status] pending</t>
         </is>
       </c>
@@ -8007,27 +8073,27 @@
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
         <is>
-          <t>Trail Side Bend Excessive</t>
+          <t>Inside Delivery</t>
         </is>
       </c>
       <c r="B29" s="13" t="inlineStr">
         <is>
-          <t>트레일측 측굴 과다</t>
+          <t>인사이드 딜리버리</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>다운스윙 중반(P6)에서 몸통의 트레일측 측면 굴곡이 정상보다 과도한 현상.</t>
+          <t>클럽이 정상보다 안쪽 경로로 접근하는 전달 패턴.</t>
         </is>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
-          <t>Thorax</t>
+          <t>Club</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Magnitude, Excessive
+          <t>Path, Inside
 [status] pending</t>
         </is>
       </c>
@@ -8035,27 +8101,27 @@
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>Handle Raise</t>
+          <t>Over The Top</t>
         </is>
       </c>
       <c r="B30" s="13" t="inlineStr">
         <is>
-          <t>핸들 상승</t>
+          <t>오버 더 탑</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>다운스윙 중반(P6)에서 그립 핸들이 정상보다 상승하는 현상.</t>
+          <t>클럽이 전달 평면 위/바깥으로 넘어가며 접근하는 패턴 (Outside Delivery 계열).</t>
         </is>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>Shaft</t>
+          <t>Club</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Motion, Raise
+          <t>Path, Outside
 [status] pending</t>
         </is>
       </c>
@@ -8063,27 +8129,27 @@
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>Handle Too Low</t>
+          <t>Trail Elbow Flying</t>
         </is>
       </c>
       <c r="B31" s="13" t="inlineStr">
         <is>
-          <t>핸들 낮음</t>
+          <t>플라잉 엘보</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>다운스윙 중반(P6)에서 그립 핸들이 정상보다 낮은 위치에 있는 현상.</t>
+          <t>트레일 팔꿈치가 몸통에서 과도하게 벌어지는(뜨는) 현상.</t>
         </is>
       </c>
       <c r="D31" s="13" t="inlineStr">
         <is>
-          <t>Shaft</t>
+          <t>Trail Elbow</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Position, Height, Low
+          <t>Position, Wide
 [status] pending</t>
         </is>
       </c>
@@ -8091,27 +8157,27 @@
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>Spine Angle Loss</t>
+          <t>Shaft Lay Down</t>
         </is>
       </c>
       <c r="B32" s="13" t="inlineStr">
         <is>
-          <t>척추각 소실</t>
+          <t>샤프트 눕힘</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>다운스윙 중반(P6)에서 어드레스에서 형성된 척추 전경각이 조기에 소실되는 현상.</t>
+          <t>샤프트가 과도하게 눕는(수평화되는) 현상. Shallow Shaft의 극단.</t>
         </is>
       </c>
       <c r="D32" s="13" t="inlineStr">
         <is>
-          <t>Spine</t>
+          <t>Shaft</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Magnitude, Loss
+          <t>Orientation, Lay Down
 [status] pending</t>
         </is>
       </c>
@@ -8119,27 +8185,27 @@
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>Chicken Wing Pattern</t>
+          <t>Handle Deep</t>
         </is>
       </c>
       <c r="B33" s="13" t="inlineStr">
         <is>
-          <t>치킨윙 패턴</t>
+          <t>핸들 깊음</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>임팩트 구간에서 리드암이 충분히 신전되지 못하고 굽혀지는 패턴. 공간·전달 실패의 보상.</t>
+          <t>그립 핸들이 정상보다 깊은(몸 뒤쪽) 위치에 있는 현상.</t>
         </is>
       </c>
       <c r="D33" s="13" t="inlineStr">
         <is>
-          <t>Arm</t>
+          <t>Shaft</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Pattern
+          <t>Position, Depth, Deep
 [status] pending</t>
         </is>
       </c>
@@ -8147,17 +8213,17 @@
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>Inside Delivery</t>
+          <t>High Angle Of Attack</t>
         </is>
       </c>
       <c r="B34" s="13" t="inlineStr">
         <is>
-          <t>인사이드 딜리버리</t>
+          <t>높은 어택앵글</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>클럽이 정상보다 안쪽 경로로 접근하는 전달 패턴.</t>
+          <t>클럽헤드가 정상보다 수직에 가까운 경로로 임팩트에 접근하는 결과.</t>
         </is>
       </c>
       <c r="D34" s="13" t="inlineStr">
@@ -8167,7 +8233,7 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Path, Inside
+          <t>Impact
 [status] pending</t>
         </is>
       </c>
@@ -8175,17 +8241,17 @@
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>Over The Top</t>
+          <t>Push Tendency</t>
         </is>
       </c>
       <c r="B35" s="13" t="inlineStr">
         <is>
-          <t>오버 더 탑</t>
+          <t>푸시 경향</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>클럽이 전달 평면 위/바깥으로 넘어가며 접근하는 패턴 (Outside Delivery 계열).</t>
+          <t>스윙 방향 대비 클럽페이스 전달이 늦어 볼이 우측으로 밀리는 경향.</t>
         </is>
       </c>
       <c r="D35" s="13" t="inlineStr">
@@ -8195,7 +8261,7 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Path, Outside
+          <t>Ball Flight
 [status] pending</t>
         </is>
       </c>
@@ -8203,27 +8269,27 @@
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>Trail Elbow Flying</t>
+          <t>Impact Consistency Decrease</t>
         </is>
       </c>
       <c r="B36" s="13" t="inlineStr">
         <is>
-          <t>플라잉 엘보</t>
+          <t>임팩트 일관성 감소</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>트레일 팔꿈치가 몸통에서 과도하게 벌어지는(뜨는) 현상.</t>
+          <t>클럽 전달이 팔 타이밍에 의존하며 임팩트 일관성이 낮아지는 결과.</t>
         </is>
       </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
-          <t>Trail Elbow</t>
+          <t>Club</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Position, Wide
+          <t>Impact
 [status] pending</t>
         </is>
       </c>
@@ -8231,27 +8297,27 @@
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>Shaft Lay Down</t>
+          <t>Lead Arm Separation Increase</t>
         </is>
       </c>
       <c r="B37" s="13" t="inlineStr">
         <is>
-          <t>샤프트 눕힘</t>
+          <t>리드암-흉곽 분리 증가</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>샤프트가 과도하게 눕는(수평화되는) 현상. Shallow Shaft의 극단.</t>
+          <t>리드암과 흉곽의 연결이 약해져 분리가 증가하는 현상.</t>
         </is>
       </c>
       <c r="D37" s="13" t="inlineStr">
         <is>
-          <t>Shaft</t>
+          <t>Arm</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>Orientation, Lay Down
+          <t>Relationship
 [status] pending</t>
         </is>
       </c>
@@ -8259,45 +8325,45 @@
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>Handle Deep</t>
+          <t>Inside Club Delivery</t>
         </is>
       </c>
       <c r="B38" s="13" t="inlineStr">
         <is>
-          <t>핸들 깊음</t>
+          <t>안쪽 전달</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>그립 핸들이 정상보다 깊은(몸 뒤쪽) 위치에 있는 현상.</t>
+          <t>클럽이 정상보다 안쪽에서 전달되는 경로. Delivery Path 축(Inside).</t>
         </is>
       </c>
       <c r="D38" s="13" t="inlineStr">
         <is>
-          <t>Shaft</t>
+          <t>Club</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>Position, Depth, Deep
-[status] pending</t>
+          <t>Delivery Path, Inside
+[status] locked-vocab</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>High Angle Of Attack</t>
+          <t>Neutral Club Delivery</t>
         </is>
       </c>
       <c r="B39" s="13" t="inlineStr">
         <is>
-          <t>높은 어택앵글</t>
+          <t>중립 전달</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>클럽헤드가 정상보다 수직에 가까운 경로로 임팩트에 접근하는 결과.</t>
+          <t>클럽 경로/플레인이 정상 범위인 상태. Delivery Path·Plane 공통 Neutral.</t>
         </is>
       </c>
       <c r="D39" s="13" t="inlineStr">
@@ -8306,166 +8372,166 @@
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Delivery Path, Plane, Neutral
+[status] locked-vocab</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>Outside Club Delivery</t>
+        </is>
+      </c>
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>바깥쪽 전달</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>클럽이 정상보다 바깥에서 전달되는 경로(out-to-in 포함). Delivery Path 축(Outside).</t>
+        </is>
+      </c>
+      <c r="D40" s="13" t="inlineStr">
+        <is>
+          <t>Club</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>Delivery Path, Outside
+[status] locked-vocab</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>Steep Club Delivery</t>
+        </is>
+      </c>
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>가파른 전달</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>클럽이 정상보다 가파른 플레인으로 전달. Delivery Plane 축(Steep).</t>
+        </is>
+      </c>
+      <c r="D41" s="13" t="inlineStr">
+        <is>
+          <t>Club</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Delivery Plane, Steep
+[status] locked-vocab</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>Shallow Club Delivery</t>
+        </is>
+      </c>
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>눕는 전달</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>클럽이 정상보다 눕는 플레인으로 전달. Delivery Plane 축(Shallow).</t>
+        </is>
+      </c>
+      <c r="D42" s="13" t="inlineStr">
+        <is>
+          <t>Club</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>Delivery Plane, Shallow
+[status] locked-vocab</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>Club Face Open At Impact</t>
+        </is>
+      </c>
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>임팩트 페이스 오픈</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>임팩트 순간 클럽페이스가 열려 있는 결과.</t>
+        </is>
+      </c>
+      <c r="D43" s="13" t="inlineStr">
+        <is>
+          <t>Club Face</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
         <is>
           <t>Impact
 [status] pending</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="13" t="inlineStr">
-        <is>
-          <t>Push Tendency</t>
-        </is>
-      </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>푸시 경향</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>스윙 방향 대비 클럽페이스 전달이 늦어 볼이 우측으로 밀리는 경향.</t>
-        </is>
-      </c>
-      <c r="D40" s="13" t="inlineStr">
-        <is>
-          <t>Club</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>Ball Flight
-[status] pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="13" t="inlineStr">
-        <is>
-          <t>Impact Consistency Decrease</t>
-        </is>
-      </c>
-      <c r="B41" s="13" t="inlineStr">
-        <is>
-          <t>임팩트 일관성 감소</t>
-        </is>
-      </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>클럽 전달이 팔 타이밍에 의존하며 임팩트 일관성이 낮아지는 결과.</t>
-        </is>
-      </c>
-      <c r="D41" s="13" t="inlineStr">
-        <is>
-          <t>Club</t>
-        </is>
-      </c>
-      <c r="E41" s="4" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="13" t="inlineStr">
+        <is>
+          <t>Club Face Closed At Impact</t>
+        </is>
+      </c>
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>임팩트 페이스 클로즈</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>임팩트 순간 클럽페이스가 닫혀 있는 결과.</t>
+        </is>
+      </c>
+      <c r="D44" s="13" t="inlineStr">
+        <is>
+          <t>Club Face</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
         <is>
           <t>Impact
 [status] pending</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="13" t="inlineStr">
-        <is>
-          <t>Lead Arm Separation Increase</t>
-        </is>
-      </c>
-      <c r="B42" s="13" t="inlineStr">
-        <is>
-          <t>리드암-흉곽 분리 증가</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>리드암과 흉곽의 연결이 약해져 분리가 증가하는 현상.</t>
-        </is>
-      </c>
-      <c r="D42" s="13" t="inlineStr">
-        <is>
-          <t>Arm</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>Relationship
-[status] pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="13" t="inlineStr">
-        <is>
-          <t>Inside Club Delivery</t>
-        </is>
-      </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t>안쪽 전달</t>
-        </is>
-      </c>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>클럽이 정상보다 안쪽에서 전달되는 경로. Delivery Path 축(Inside).</t>
-        </is>
-      </c>
-      <c r="D43" s="13" t="inlineStr">
-        <is>
-          <t>Club</t>
-        </is>
-      </c>
-      <c r="E43" s="4" t="inlineStr">
-        <is>
-          <t>Delivery Path, Inside
-[status] locked-vocab</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="13" t="inlineStr">
-        <is>
-          <t>Neutral Club Delivery</t>
-        </is>
-      </c>
-      <c r="B44" s="13" t="inlineStr">
-        <is>
-          <t>중립 전달</t>
-        </is>
-      </c>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>클럽 경로/플레인이 정상 범위인 상태. Delivery Path·Plane 공통 Neutral.</t>
-        </is>
-      </c>
-      <c r="D44" s="13" t="inlineStr">
-        <is>
-          <t>Club</t>
-        </is>
-      </c>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t>Delivery Path, Plane, Neutral
-[status] locked-vocab</t>
-        </is>
-      </c>
-    </row>
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>Outside Club Delivery</t>
+          <t>Reduced Club Control</t>
         </is>
       </c>
       <c r="B45" s="13" t="inlineStr">
         <is>
-          <t>바깥쪽 전달</t>
+          <t>클럽 컨트롤 저하</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>클럽이 정상보다 바깥에서 전달되는 경로(out-to-in 포함). Delivery Path 축(Outside).</t>
+          <t>팔 타이밍 의존 등으로 클럽 컨트롤·일관성이 낮아지는 결과.</t>
         </is>
       </c>
       <c r="D45" s="13" t="inlineStr">
@@ -8475,153 +8541,265 @@
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>Delivery Path, Outside
-[status] locked-vocab</t>
+          <t>Impact
+[status] pending</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>Steep Club Delivery</t>
+          <t>Early Upper Body Rotation</t>
         </is>
       </c>
       <c r="B46" s="13" t="inlineStr">
         <is>
-          <t>가파른 전달</t>
+          <t>상체 조기 회전</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>클럽이 정상보다 가파른 플레인으로 전달. Delivery Plane 축(Steep).</t>
+          <t>팔 전달보다 상체가 먼저 회전하는 Prediction 링크.</t>
         </is>
       </c>
       <c r="D46" s="13" t="inlineStr">
         <is>
-          <t>Club</t>
+          <t>Thorax</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Delivery Plane, Steep
-[status] locked-vocab</t>
+          <t>Prediction
+[status] prediction-vocab</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>Shallow Club Delivery</t>
+          <t>Blocked Body Rotation</t>
         </is>
       </c>
       <c r="B47" s="13" t="inlineStr">
         <is>
-          <t>눕는 전달</t>
+          <t>몸통 회전 막힘</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>클럽이 정상보다 눕는 플레인으로 전달. Delivery Plane 축(Shallow).</t>
+          <t>몸통 회전이 정체·차단되는 Prediction 링크.</t>
         </is>
       </c>
       <c r="D47" s="13" t="inlineStr">
         <is>
-          <t>Club</t>
+          <t>Thorax</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>Delivery Plane, Shallow
-[status] locked-vocab</t>
+          <t>Prediction
+[status] prediction-vocab</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>Club Face Open At Impact</t>
+          <t>Trail Elbow Tucked</t>
         </is>
       </c>
       <c r="B48" s="13" t="inlineStr">
         <is>
-          <t>임팩트 페이스 오픈</t>
+          <t>트레일 팔꿈치 붙음</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>임팩트 순간 클럽페이스가 열려 있는 결과.</t>
+          <t>트레일 팔꿈치가 몸통에 붙어 인사이드 전달을 만드는 링크(훅 계열).</t>
         </is>
       </c>
       <c r="D48" s="13" t="inlineStr">
         <is>
-          <t>Club Face</t>
+          <t>Trail Elbow</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>Impact
-[status] pending</t>
+          <t>Prediction
+[status] prediction-vocab</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>Club Face Closed At Impact</t>
+          <t>Reduced Lag</t>
         </is>
       </c>
       <c r="B49" s="13" t="inlineStr">
         <is>
-          <t>임팩트 페이스 클로즈</t>
+          <t>래그 감소</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>임팩트 순간 클럽페이스가 닫혀 있는 결과.</t>
+          <t>래그가 조기 소실되는 Prediction 링크.</t>
         </is>
       </c>
       <c r="D49" s="13" t="inlineStr">
         <is>
-          <t>Club Face</t>
+          <t>Club</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>Impact
-[status] pending</t>
+          <t>Prediction
+[status] prediction-vocab</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>Reduced Club Control</t>
+          <t>Thoracic Hyperextension</t>
         </is>
       </c>
       <c r="B50" s="13" t="inlineStr">
         <is>
-          <t>클럽 컨트롤 저하</t>
+          <t>흉추 과신전</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>팔 타이밍 의존 등으로 클럽 컨트롤·일관성이 낮아지는 결과.</t>
+          <t>흉추가 과신전되는 링크(Cross Line 계열).</t>
         </is>
       </c>
       <c r="D50" s="13" t="inlineStr">
         <is>
-          <t>Club</t>
+          <t>Spine</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>Impact
-[status] pending</t>
+          <t>Prediction
+[status] prediction-vocab</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>Increased Vertical Force</t>
+        </is>
+      </c>
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>수직력 증가</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>지면반력 수직 성분이 증가하는 링크(Head Drop 계열).</t>
+        </is>
+      </c>
+      <c r="D51" s="13" t="inlineStr">
+        <is>
+          <t>Pressure</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>Prediction
+[status] prediction-vocab</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="13" t="inlineStr">
+        <is>
+          <t>Side Bend Compensation</t>
+        </is>
+      </c>
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>측굴 보상</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>측굴로 전달을 보상하는 링크.</t>
+        </is>
+      </c>
+      <c r="D52" s="13" t="inlineStr">
+        <is>
+          <t>Thorax</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>Prediction
+[status] prediction-vocab</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="13" t="inlineStr">
+        <is>
+          <t>Excessive Side Bend</t>
+        </is>
+      </c>
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>과도한 측굴</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>트레일측 측굴이 과도한 링크.</t>
+        </is>
+      </c>
+      <c r="D53" s="13" t="inlineStr">
+        <is>
+          <t>Thorax</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>Prediction
+[status] prediction-vocab</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="13" t="inlineStr">
+        <is>
+          <t>Trail Arm Extension Compensation</t>
+        </is>
+      </c>
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>트레일 팔 신전 보상</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>트레일 팔을 펴 인사이드 전달을 보상하는 링크.</t>
+        </is>
+      </c>
+      <c r="D54" s="13" t="inlineStr">
+        <is>
+          <t>Arm</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>Prediction
+[status] prediction-vocab</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E50"/>
+  <autoFilter ref="A1:E54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8632,7 +8810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:O37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -9311,7 +9489,7 @@
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t>Late Trail Foot Release</t>
+          <t>Cross-over Top Pattern</t>
         </is>
       </c>
       <c r="B25" s="14" t="n"/>
@@ -9332,7 +9510,7 @@
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>Left Start Direction</t>
+          <t>Spine Flexion Excessive</t>
         </is>
       </c>
       <c r="B26" s="14" t="n"/>
@@ -9353,7 +9531,7 @@
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t>Cross-over Top Pattern</t>
+          <t>Trail Side Bend Excessive</t>
         </is>
       </c>
       <c r="B27" s="14" t="n"/>
@@ -9374,7 +9552,7 @@
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t>Spine Flexion Excessive</t>
+          <t>Chicken Wing Pattern</t>
         </is>
       </c>
       <c r="B28" s="14" t="n"/>
@@ -9395,7 +9573,7 @@
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
         <is>
-          <t>Trail Side Bend Excessive</t>
+          <t>Inside Delivery</t>
         </is>
       </c>
       <c r="B29" s="14" t="n"/>
@@ -9416,7 +9594,7 @@
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>Handle Raise</t>
+          <t>Over The Top</t>
         </is>
       </c>
       <c r="B30" s="14" t="n"/>
@@ -9437,7 +9615,7 @@
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>Handle Too Low</t>
+          <t>Trail Elbow Flying</t>
         </is>
       </c>
       <c r="B31" s="14" t="n"/>
@@ -9458,7 +9636,7 @@
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>Spine Angle Loss</t>
+          <t>Shaft Lay Down</t>
         </is>
       </c>
       <c r="B32" s="14" t="n"/>
@@ -9479,7 +9657,7 @@
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>Chicken Wing Pattern</t>
+          <t>Handle Deep</t>
         </is>
       </c>
       <c r="B33" s="14" t="n"/>
@@ -9500,7 +9678,7 @@
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>Inside Delivery</t>
+          <t>High Angle Of Attack</t>
         </is>
       </c>
       <c r="B34" s="14" t="n"/>
@@ -9521,7 +9699,7 @@
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>Over The Top</t>
+          <t>Push Tendency</t>
         </is>
       </c>
       <c r="B35" s="14" t="n"/>
@@ -9542,7 +9720,7 @@
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>Trail Elbow Flying</t>
+          <t>Impact Consistency Decrease</t>
         </is>
       </c>
       <c r="B36" s="14" t="n"/>
@@ -9563,7 +9741,7 @@
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>Shaft Lay Down</t>
+          <t>Lead Arm Separation Increase</t>
         </is>
       </c>
       <c r="B37" s="14" t="n"/>
@@ -9581,113 +9759,8 @@
       <c r="N37" s="14" t="n"/>
       <c r="O37" s="14" t="n"/>
     </row>
-    <row r="38">
-      <c r="A38" s="13" t="inlineStr">
-        <is>
-          <t>Handle Deep</t>
-        </is>
-      </c>
-      <c r="B38" s="14" t="n"/>
-      <c r="C38" s="14" t="n"/>
-      <c r="D38" s="14" t="n"/>
-      <c r="E38" s="14" t="n"/>
-      <c r="F38" s="14" t="n"/>
-      <c r="G38" s="14" t="n"/>
-      <c r="H38" s="14" t="n"/>
-      <c r="I38" s="14" t="n"/>
-      <c r="J38" s="14" t="n"/>
-      <c r="K38" s="14" t="n"/>
-      <c r="L38" s="14" t="n"/>
-      <c r="M38" s="14" t="n"/>
-      <c r="N38" s="14" t="n"/>
-      <c r="O38" s="14" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="13" t="inlineStr">
-        <is>
-          <t>High Angle Of Attack</t>
-        </is>
-      </c>
-      <c r="B39" s="14" t="n"/>
-      <c r="C39" s="14" t="n"/>
-      <c r="D39" s="14" t="n"/>
-      <c r="E39" s="14" t="n"/>
-      <c r="F39" s="14" t="n"/>
-      <c r="G39" s="14" t="n"/>
-      <c r="H39" s="14" t="n"/>
-      <c r="I39" s="14" t="n"/>
-      <c r="J39" s="14" t="n"/>
-      <c r="K39" s="14" t="n"/>
-      <c r="L39" s="14" t="n"/>
-      <c r="M39" s="14" t="n"/>
-      <c r="N39" s="14" t="n"/>
-      <c r="O39" s="14" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="13" t="inlineStr">
-        <is>
-          <t>Push Tendency</t>
-        </is>
-      </c>
-      <c r="B40" s="14" t="n"/>
-      <c r="C40" s="14" t="n"/>
-      <c r="D40" s="14" t="n"/>
-      <c r="E40" s="14" t="n"/>
-      <c r="F40" s="14" t="n"/>
-      <c r="G40" s="14" t="n"/>
-      <c r="H40" s="14" t="n"/>
-      <c r="I40" s="14" t="n"/>
-      <c r="J40" s="14" t="n"/>
-      <c r="K40" s="14" t="n"/>
-      <c r="L40" s="14" t="n"/>
-      <c r="M40" s="14" t="n"/>
-      <c r="N40" s="14" t="n"/>
-      <c r="O40" s="14" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="13" t="inlineStr">
-        <is>
-          <t>Impact Consistency Decrease</t>
-        </is>
-      </c>
-      <c r="B41" s="14" t="n"/>
-      <c r="C41" s="14" t="n"/>
-      <c r="D41" s="14" t="n"/>
-      <c r="E41" s="14" t="n"/>
-      <c r="F41" s="14" t="n"/>
-      <c r="G41" s="14" t="n"/>
-      <c r="H41" s="14" t="n"/>
-      <c r="I41" s="14" t="n"/>
-      <c r="J41" s="14" t="n"/>
-      <c r="K41" s="14" t="n"/>
-      <c r="L41" s="14" t="n"/>
-      <c r="M41" s="14" t="n"/>
-      <c r="N41" s="14" t="n"/>
-      <c r="O41" s="14" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="13" t="inlineStr">
-        <is>
-          <t>Lead Arm Separation Increase</t>
-        </is>
-      </c>
-      <c r="B42" s="14" t="n"/>
-      <c r="C42" s="14" t="n"/>
-      <c r="D42" s="14" t="n"/>
-      <c r="E42" s="14" t="n"/>
-      <c r="F42" s="14" t="n"/>
-      <c r="G42" s="14" t="n"/>
-      <c r="H42" s="14" t="n"/>
-      <c r="I42" s="14" t="n"/>
-      <c r="J42" s="14" t="n"/>
-      <c r="K42" s="14" t="n"/>
-      <c r="L42" s="14" t="n"/>
-      <c r="M42" s="14" t="n"/>
-      <c r="N42" s="14" t="n"/>
-      <c r="O42" s="14" t="n"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:O42"/>
+  <autoFilter ref="A1:O37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix(P6): Evidence Matrix 소스를 최신 업로드로 수정 (Casting/Spin-out 등 수치 누락 버그)
빌드 스크립트가 이전 업로드(9f8581fd-DOH_P6.xlsx)를 계속 참조하고 있어,
그 이후 업로드(e518f8a3-DOH_P6_1.xlsx)에 추가로 채워진 Evidence Matrix
수치(Casting/Spin-out/Late Arm/Trail Elbow/Steep·Shallow Shaft/Lead Pressure 등)가
반영되지 않고 있었음. 소스를 최신 업로드로 교체.

여전히 비어있는 5개(정상, 수치 미제공): Pelvis Stall, Thorax Rotation Excessive,
Hands Too Close/Far From Body, Incomplete Pressure Transfer

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015JSgPBxwLoJqyCWhXnBVL3
</commit_message>
<xml_diff>
--- a/DOH_P6.xlsx
+++ b/DOH_P6.xlsx
@@ -9265,12 +9265,24 @@
       <c r="C14" s="14" t="n"/>
       <c r="D14" s="14" t="n"/>
       <c r="E14" s="14" t="n"/>
-      <c r="F14" s="14" t="n"/>
-      <c r="G14" s="14" t="n"/>
-      <c r="H14" s="14" t="n"/>
-      <c r="I14" s="14" t="n"/>
-      <c r="J14" s="14" t="n"/>
-      <c r="K14" s="14" t="n"/>
+      <c r="F14" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H14" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="I14" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="J14" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="K14" s="14" t="n">
+        <v>3</v>
+      </c>
       <c r="L14" s="14" t="n"/>
       <c r="M14" s="14" t="n"/>
       <c r="N14" s="14" t="n"/>
@@ -9286,12 +9298,24 @@
       <c r="C15" s="14" t="n"/>
       <c r="D15" s="14" t="n"/>
       <c r="E15" s="14" t="n"/>
-      <c r="F15" s="14" t="n"/>
-      <c r="G15" s="14" t="n"/>
-      <c r="H15" s="14" t="n"/>
-      <c r="I15" s="14" t="n"/>
-      <c r="J15" s="14" t="n"/>
-      <c r="K15" s="14" t="n"/>
+      <c r="F15" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="G15" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H15" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="I15" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="J15" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="K15" s="14" t="n">
+        <v>4</v>
+      </c>
       <c r="L15" s="14" t="n"/>
       <c r="M15" s="14" t="n"/>
       <c r="N15" s="14" t="n"/>
@@ -9307,12 +9331,24 @@
       <c r="C16" s="14" t="n"/>
       <c r="D16" s="14" t="n"/>
       <c r="E16" s="14" t="n"/>
-      <c r="F16" s="14" t="n"/>
-      <c r="G16" s="14" t="n"/>
-      <c r="H16" s="14" t="n"/>
-      <c r="I16" s="14" t="n"/>
-      <c r="J16" s="14" t="n"/>
-      <c r="K16" s="14" t="n"/>
+      <c r="F16" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="G16" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H16" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="I16" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="J16" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="K16" s="14" t="n">
+        <v>3</v>
+      </c>
       <c r="L16" s="14" t="n"/>
       <c r="M16" s="14" t="n"/>
       <c r="N16" s="14" t="n"/>
@@ -9328,12 +9364,24 @@
       <c r="C17" s="14" t="n"/>
       <c r="D17" s="14" t="n"/>
       <c r="E17" s="14" t="n"/>
-      <c r="F17" s="14" t="n"/>
-      <c r="G17" s="14" t="n"/>
-      <c r="H17" s="14" t="n"/>
-      <c r="I17" s="14" t="n"/>
-      <c r="J17" s="14" t="n"/>
-      <c r="K17" s="14" t="n"/>
+      <c r="F17" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H17" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="I17" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="J17" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="K17" s="14" t="n">
+        <v>4</v>
+      </c>
       <c r="L17" s="14" t="n"/>
       <c r="M17" s="14" t="n"/>
       <c r="N17" s="14" t="n"/>
@@ -9349,12 +9397,24 @@
       <c r="C18" s="14" t="n"/>
       <c r="D18" s="14" t="n"/>
       <c r="E18" s="14" t="n"/>
-      <c r="F18" s="14" t="n"/>
-      <c r="G18" s="14" t="n"/>
-      <c r="H18" s="14" t="n"/>
-      <c r="I18" s="14" t="n"/>
-      <c r="J18" s="14" t="n"/>
-      <c r="K18" s="14" t="n"/>
+      <c r="F18" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H18" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="I18" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="J18" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="K18" s="14" t="n">
+        <v>3</v>
+      </c>
       <c r="L18" s="14" t="n"/>
       <c r="M18" s="14" t="n"/>
       <c r="N18" s="14" t="n"/>
@@ -9370,12 +9430,24 @@
       <c r="C19" s="14" t="n"/>
       <c r="D19" s="14" t="n"/>
       <c r="E19" s="14" t="n"/>
-      <c r="F19" s="14" t="n"/>
-      <c r="G19" s="14" t="n"/>
-      <c r="H19" s="14" t="n"/>
-      <c r="I19" s="14" t="n"/>
-      <c r="J19" s="14" t="n"/>
-      <c r="K19" s="14" t="n"/>
+      <c r="F19" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="G19" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H19" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="I19" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="J19" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="K19" s="14" t="n">
+        <v>3</v>
+      </c>
       <c r="L19" s="14" t="n"/>
       <c r="M19" s="14" t="n"/>
       <c r="N19" s="14" t="n"/>
@@ -9391,12 +9463,24 @@
       <c r="C20" s="14" t="n"/>
       <c r="D20" s="14" t="n"/>
       <c r="E20" s="14" t="n"/>
-      <c r="F20" s="14" t="n"/>
-      <c r="G20" s="14" t="n"/>
-      <c r="H20" s="14" t="n"/>
-      <c r="I20" s="14" t="n"/>
-      <c r="J20" s="14" t="n"/>
-      <c r="K20" s="14" t="n"/>
+      <c r="F20" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="G20" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H20" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="I20" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="J20" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="K20" s="14" t="n">
+        <v>4</v>
+      </c>
       <c r="L20" s="14" t="n"/>
       <c r="M20" s="14" t="n"/>
       <c r="N20" s="14" t="n"/>
@@ -9433,12 +9517,24 @@
       <c r="C22" s="14" t="n"/>
       <c r="D22" s="14" t="n"/>
       <c r="E22" s="14" t="n"/>
-      <c r="F22" s="14" t="n"/>
-      <c r="G22" s="14" t="n"/>
-      <c r="H22" s="14" t="n"/>
-      <c r="I22" s="14" t="n"/>
-      <c r="J22" s="14" t="n"/>
-      <c r="K22" s="14" t="n"/>
+      <c r="F22" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="G22" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H22" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="I22" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="J22" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="K22" s="14" t="n">
+        <v>2</v>
+      </c>
       <c r="L22" s="14" t="n"/>
       <c r="M22" s="14" t="n"/>
       <c r="N22" s="14" t="n"/>
@@ -9496,12 +9592,24 @@
       <c r="C25" s="14" t="n"/>
       <c r="D25" s="14" t="n"/>
       <c r="E25" s="14" t="n"/>
-      <c r="F25" s="14" t="n"/>
-      <c r="G25" s="14" t="n"/>
-      <c r="H25" s="14" t="n"/>
-      <c r="I25" s="14" t="n"/>
-      <c r="J25" s="14" t="n"/>
-      <c r="K25" s="14" t="n"/>
+      <c r="F25" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="G25" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H25" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="I25" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="J25" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="K25" s="14" t="n">
+        <v>3</v>
+      </c>
       <c r="L25" s="14" t="n"/>
       <c r="M25" s="14" t="n"/>
       <c r="N25" s="14" t="n"/>
@@ -9559,12 +9667,24 @@
       <c r="C28" s="14" t="n"/>
       <c r="D28" s="14" t="n"/>
       <c r="E28" s="14" t="n"/>
-      <c r="F28" s="14" t="n"/>
-      <c r="G28" s="14" t="n"/>
-      <c r="H28" s="14" t="n"/>
-      <c r="I28" s="14" t="n"/>
-      <c r="J28" s="14" t="n"/>
-      <c r="K28" s="14" t="n"/>
+      <c r="F28" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="G28" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H28" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="I28" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="J28" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="K28" s="14" t="n">
+        <v>3</v>
+      </c>
       <c r="L28" s="14" t="n"/>
       <c r="M28" s="14" t="n"/>
       <c r="N28" s="14" t="n"/>

</xml_diff>